<commit_message>
Follow-ups: donor entry backups and restore, one home for donor data, pyxform tests
- Automatic dated backups of entries.db (every save, import and dashboard start; newest 30),
  "Download backup" Excel export, restore command (backs up the current file first); tested
- One-time "Import from the Excel tracker" with preview and confirmation: keeps IDs and
  origin file/sheet/row; the pipeline stops reading imported Excel rows; individual donor
  labels and donor keys unchanged; donor template kept as an offline fallback
- pyxform 4.5.0 in requirements-dev.txt; the Kobo forms are converted in the tests
- Limitations (no login, single laptop, Kobo unchecked), partner questions F7/F8 expanded
- Decision log D200-D205; instruction log entry 13

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/donor_opportunity_template.xlsx
+++ b/templates/donor_opportunity_template.xlsx
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -589,240 +589,247 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>- OFFLINE FALLBACK ONLY. Donor data is kept on the dashboard's Donor entry page. Use this file only when the dashboard cannot be used (for example away from the office laptop), for NEW opportunities with NEW IDs; import them on the Donor entry page afterwards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>- Opportunities sheet: one row per funding opportunity (a call, a proposal, a renewal). Keep the row when it is won or lost: change the Stage.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>- Stages, in order: Identified (we know about it) - Qualified (we fit and decided to go) - Concept note - Proposal submitted - then the OUTCOME: Awarded or Declined.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>- Probability: your honest guess that it will be awarded, as a percentage (type 40% or 0.4). The dashboard multiplies the amount requested by it (the 'weighted' value). Declined = 0%; Awarded = 100%.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>- Amounts in RWF, numbers only (no 'RWF', no commas). When the Stage is Awarded, fill in the Awarded amount.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>- Thematic fit: pick WASH, Agriculture or both ('WASH; Agriculture'). An opportunity that fits both is split half and half between the themes on the dashboard.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>- Next action and its date: the one thing to do next, and by when. Dates in the past show in red here and in the 'Overdue next actions' list on the dashboard.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>- Colours on the Opportunities sheet: red = next action overdue; amber = deadline within 30 days; orange = Awarded with no awarded amount.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="n"/>
-    </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Orange headers are required. Do not rename, reorder or delete columns.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Example rows (for illustration only: type real rows on the Opportunities sheet)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Opp ID</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Opportunity title</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Donor</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>Thematic fit</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>Deadline</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>Requested amount (RWF)</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>Awarded amount (RWF)</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>Probability</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="K18" s="5" t="inlineStr">
         <is>
           <t>Next action</t>
         </is>
       </c>
-      <c r="L17" s="5" t="inlineStr">
+      <c r="L18" s="5" t="inlineStr">
         <is>
           <t>Next action date</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>OPP001</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Safe water for schools - Kayonza</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Example Foundation</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>WASH</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Concept note</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>30/09/2026</t>
         </is>
       </c>
-      <c r="G18" t="n">
+      <c r="G19" t="n">
         <v>150000000</v>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>ED</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>Send concept note</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>15/08/2026</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>OPP002</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Climate-smart farming phase 2</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Example Bilateral Agency</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Awarded</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>01/03/2026</t>
         </is>
       </c>
-      <c r="G19" t="n">
+      <c r="G20" t="n">
         <v>200000000</v>
       </c>
-      <c r="H19" t="n">
+      <c r="H20" t="n">
         <v>180000000</v>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>PM01</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>Sign grant agreement</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>10/07/2026</t>
         </is>

</xml_diff>